<commit_message>
Studied theory of disjoint sets
</commit_message>
<xml_diff>
--- a/DSA.xlsx
+++ b/DSA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\2026\learninglog\DSA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82414212-B978-4B9C-9A31-A2A6C49AE4CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A9F48BD-61B5-4780-8D52-BAE67E9BC757}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,14 +18,16 @@
     <sheet name="Recurrsion" sheetId="3" r:id="rId3"/>
     <sheet name="Tree" sheetId="4" r:id="rId4"/>
     <sheet name="Graph" sheetId="5" r:id="rId5"/>
-    <sheet name="LinkedList" sheetId="6" r:id="rId6"/>
-    <sheet name="Subarray" sheetId="8" r:id="rId7"/>
-    <sheet name="Sliding Window" sheetId="7" r:id="rId8"/>
+    <sheet name="Bitmanupulation" sheetId="9" r:id="rId6"/>
+    <sheet name="LinkedList" sheetId="6" r:id="rId7"/>
+    <sheet name="Subarray" sheetId="8" r:id="rId8"/>
+    <sheet name="Sliding Window" sheetId="7" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Graph!$A$1:$N$27</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Sliding Window'!$A$1:$O$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">Subarray!$A$1:$N$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Bitmanupulation!$A$1:$O$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Graph!$A$1:$N$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Sliding Window'!$A$1:$O$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">Subarray!$A$1:$N$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="467" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="508" uniqueCount="254">
   <si>
     <t xml:space="preserve">Problem Name </t>
   </si>
@@ -1639,9 +1641,6 @@
       </rPr>
       <t>No need to use visited array to prevent mutiple updates for already visited cell . we can use distance from that as well .</t>
     </r>
-  </si>
-  <si>
-    <t>#1</t>
   </si>
   <si>
     <t>Revision (#1-26-01-25)</t>
@@ -2011,73 +2010,6 @@
     </r>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">NEED : </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Dijkstra don't work on negative edges and gives tle in case of negative cycle in the graph . 
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>APPROCH :</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> 
-- Intialize the cost with MAX except Source node .
-- Iterate over the edges totalnodes-1 times and update cost array for the node if we can reach it with minimum cost than previous.
-- while Iterating on edges Nth time if we find any updation then return saying "Cycle exists in the graph".
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFFC000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>NOTES :</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Cycle in a graph which contain at least one negative edge doesn't means negative cycle . Sum of the cycle path must be less than zero to say "Negative Cycle".</t>
-    </r>
-  </si>
-  <si>
     <t>https://takeuforward.org/data-structure/floyd-warshall-algorithm-g-42</t>
   </si>
   <si>
@@ -2207,12 +2139,171 @@
     <t>TC - O(n^3)
 SC - O(n)</t>
   </si>
+  <si>
+    <t>696. Count Binary Substrings</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/count-binary-substrings</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/count-binary-substrings/solutions/7590577/count-binary-substrings-easy-solution-by-it1w/?envType=daily-question&amp;envId=2026-02-19</t>
+  </si>
+  <si>
+    <t>TC - O(n)</t>
+  </si>
+  <si>
+    <t>Bitmanupulation</t>
+  </si>
+  <si>
+    <t>POTD</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">NEED : </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Dijkstra don't work on negative edges and gives tle in case of negative cycle in the graph . 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>APPROCH :</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 
+- Intialize the cost with MAX except Source node .
+- Iterate over the edges totalnodes-1 times and update cost array for the node if we can reach it with minimum cost than previous.
+- while Iterating on edges Nth time if we find any updation then return saying "Negative Cycle exists in the graph".
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFFC000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>NOTES :</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Cycle in a graph which contain at least one negative edge doesn't means negative cycle . Sum of the cycle path must be less than zero to say "Negative Cycle".</t>
+    </r>
+  </si>
+  <si>
+    <t>#1-09-03-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  </t>
+  </si>
+  <si>
+    <t>#1-11-03-26</t>
+  </si>
+  <si>
+    <t>MST - Prims Algo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Medium </t>
+  </si>
+  <si>
+    <t xml:space="preserve">yes - </t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC - O(E log V) </t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">NEED :  To find minimum spanning tree . 
+Maintain a sum variable and list to maintain Min. sum and pair of the mst.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="9"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Algorithum :</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 
+1. Initialize the visited array and priority queue - (weight,node,parent).
+2. Add any node as starting node with (0,node ,-1).
+3. while q is not empty 
+3.1 poll the peek of pq , if it's not already been visited, mark it as visited .
+3.2 explore its adjacent , if adjancent is not visited  and add in the queue .
+4 repeat </t>
+    </r>
+  </si>
+  <si>
+    <t>1584. Min Cost to Connect All Points</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/min-cost-to-connect-all-points/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Intution : If we represent (x,y) as vertex , then problem comes down to MST by prims . 
+Hint : As all  (x,y) are unique we can consider points.length == no. vertexs and we will calculate distance between them as weight . 
+Approch : represent each (x,y) vertex and create adjacency list with everyother vertex . </t>
+  </si>
+  <si>
+    <t>TC - O(n^2 log n)</t>
+  </si>
+  <si>
+    <t>MST Prim's algo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Disjoint Set By Rank and Size </t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2266,6 +2357,13 @@
     <font>
       <sz val="11"/>
       <color rgb="FF7030A0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="9"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -2971,7 +3069,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{627F4D11-A7C4-43BB-9B31-F105D2E4CA7B}">
-  <dimension ref="A1:O31"/>
+  <dimension ref="A1:O34"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="25.90625" style="5" customWidth="1"/>
@@ -3014,7 +3112,7 @@
         <v>140</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="J1" s="5" t="s">
         <v>44</v>
@@ -3058,7 +3156,7 @@
         <v>5</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="J2" s="5" t="s">
         <v>77</v>
@@ -3096,7 +3194,7 @@
         <v>5</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="J3" s="5" t="s">
         <v>80</v>
@@ -3131,7 +3229,7 @@
         <v>5</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="J4" s="5" t="s">
         <v>79</v>
@@ -3166,7 +3264,7 @@
         <v>4</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="K5" s="9" t="s">
         <v>49</v>
@@ -3201,7 +3299,7 @@
         <v>5</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="K6" s="9" t="s">
         <v>49</v>
@@ -3236,7 +3334,7 @@
         <v>4</v>
       </c>
       <c r="I7" s="5" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="J7" s="5" t="s">
         <v>84</v>
@@ -3256,7 +3354,7 @@
         <v>62</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>82</v>
@@ -3667,7 +3765,7 @@
         <v>3</v>
       </c>
       <c r="I20" s="5" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="K20" s="9" t="s">
         <v>32</v>
@@ -3757,7 +3855,7 @@
         <v>179</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="E23" s="9" t="s">
         <v>32</v>
@@ -3875,7 +3973,7 @@
       <c r="A27" s="5" t="s">
         <v>190</v>
       </c>
-      <c r="B27" s="5" t="s">
+      <c r="B27" s="7" t="s">
         <v>191</v>
       </c>
       <c r="C27" s="5" t="s">
@@ -3897,7 +3995,7 @@
         <v>4</v>
       </c>
       <c r="I27" s="5" t="s">
-        <v>196</v>
+        <v>242</v>
       </c>
       <c r="K27" s="9" t="s">
         <v>32</v>
@@ -3911,22 +4009,22 @@
     </row>
     <row r="28" spans="1:13" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A28" s="5" t="s">
+        <v>200</v>
+      </c>
+      <c r="B28" s="7" t="s">
         <v>201</v>
       </c>
-      <c r="B28" s="7" t="s">
+      <c r="C28" s="5" t="s">
+        <v>204</v>
+      </c>
+      <c r="D28" s="5" t="s">
         <v>202</v>
-      </c>
-      <c r="C28" s="5" t="s">
-        <v>205</v>
-      </c>
-      <c r="D28" s="5" t="s">
-        <v>203</v>
       </c>
       <c r="E28" s="9" t="s">
         <v>25</v>
       </c>
       <c r="F28" s="9" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="G28" s="5" t="s">
         <v>194</v>
@@ -3934,6 +4032,9 @@
       <c r="H28" s="5">
         <v>3</v>
       </c>
+      <c r="I28" s="5" t="s">
+        <v>240</v>
+      </c>
       <c r="K28" s="9" t="s">
         <v>32</v>
       </c>
@@ -3946,16 +4047,16 @@
     </row>
     <row r="29" spans="1:13" ht="362.5" x14ac:dyDescent="0.35">
       <c r="A29" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="B29" s="7" t="s">
         <v>211</v>
       </c>
-      <c r="B29" s="7" t="s">
+      <c r="C29" s="5" t="s">
+        <v>239</v>
+      </c>
+      <c r="D29" s="5" t="s">
         <v>212</v>
-      </c>
-      <c r="C29" s="5" t="s">
-        <v>226</v>
-      </c>
-      <c r="D29" s="5" t="s">
-        <v>213</v>
       </c>
       <c r="E29" s="9" t="s">
         <v>25</v>
@@ -3964,27 +4065,30 @@
         <v>66</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="H29" s="5">
         <v>4</v>
       </c>
+      <c r="I29" s="5" t="s">
+        <v>241</v>
+      </c>
       <c r="J29" s="5" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="30" spans="1:13" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A30" s="5" t="s">
+        <v>226</v>
+      </c>
+      <c r="B30" s="7" t="s">
+        <v>225</v>
+      </c>
+      <c r="C30" s="11" t="s">
+        <v>227</v>
+      </c>
+      <c r="D30" s="5" t="s">
         <v>228</v>
-      </c>
-      <c r="B30" s="7" t="s">
-        <v>227</v>
-      </c>
-      <c r="C30" s="11" t="s">
-        <v>229</v>
-      </c>
-      <c r="D30" s="5" t="s">
-        <v>230</v>
       </c>
       <c r="E30" s="9" t="s">
         <v>32</v>
@@ -3996,21 +4100,21 @@
         <v>3</v>
       </c>
       <c r="J30" s="5" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="31" spans="1:13" ht="261" x14ac:dyDescent="0.35">
       <c r="A31" s="5" t="s">
+        <v>229</v>
+      </c>
+      <c r="B31" s="7" t="s">
+        <v>230</v>
+      </c>
+      <c r="C31" s="5" t="s">
         <v>231</v>
       </c>
-      <c r="B31" s="5" t="s">
+      <c r="D31" s="5" t="s">
         <v>232</v>
-      </c>
-      <c r="C31" s="5" t="s">
-        <v>233</v>
-      </c>
-      <c r="D31" s="5" t="s">
-        <v>234</v>
       </c>
       <c r="E31" s="9" t="s">
         <v>25</v>
@@ -4019,17 +4123,80 @@
         <v>43</v>
       </c>
       <c r="G31" s="5" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="H31" s="5">
         <v>4</v>
       </c>
+      <c r="I31" s="5" t="s">
+        <v>240</v>
+      </c>
       <c r="M31" s="5" t="s">
-        <v>228</v>
+        <v>226</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" ht="275.5" x14ac:dyDescent="0.35">
+      <c r="A32" s="5" t="s">
+        <v>243</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>247</v>
+      </c>
+      <c r="D32" s="5" t="s">
+        <v>246</v>
+      </c>
+      <c r="F32" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="H32" s="5">
+        <v>3</v>
+      </c>
+      <c r="J32" s="5" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13" ht="188.5" x14ac:dyDescent="0.35">
+      <c r="A33" s="5" t="s">
+        <v>248</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>249</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>250</v>
+      </c>
+      <c r="D33" s="5" t="s">
+        <v>251</v>
+      </c>
+      <c r="E33" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="F33" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="G33" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="H33" s="5">
+        <v>3</v>
+      </c>
+      <c r="K33" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="L33" s="5" t="s">
+        <v>243</v>
+      </c>
+      <c r="M33" s="5" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A34" s="5" t="s">
+        <v>253</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N27" xr:uid="{627F4D11-A7C4-43BB-9B31-F105D2E4CA7B}"/>
+  <autoFilter ref="A1:N32" xr:uid="{627F4D11-A7C4-43BB-9B31-F105D2E4CA7B}"/>
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1" display="https://takeuforward.org/plus/dsa/problems/connected-components" xr:uid="{CBDDA4D9-3DA6-42F4-BD81-6766CE6059E4}"/>
     <hyperlink ref="B4" r:id="rId2" xr:uid="{D4ED72D4-0FD6-484E-AD61-CDBC7D2FE01F}"/>
@@ -4052,13 +4219,119 @@
     <hyperlink ref="B28" r:id="rId19" xr:uid="{5CEB0A28-62E3-4F7D-9DA7-371B1C990640}"/>
     <hyperlink ref="B29" r:id="rId20" xr:uid="{ED6D3629-9BAC-4F79-9135-D4EA70CC2E96}"/>
     <hyperlink ref="B30" r:id="rId21" xr:uid="{6A758F7A-79FB-495C-B418-9EDF46598B5E}"/>
+    <hyperlink ref="B31" r:id="rId22" xr:uid="{3472C449-0813-4249-A912-7371C1132D75}"/>
+    <hyperlink ref="B27" r:id="rId23" xr:uid="{E7B363CE-2ADD-4EB8-BDCC-4504C7B2FC63}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId22"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId24"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD994AD9-DD9F-4AD2-9BE6-CF2C5785A85E}">
+  <dimension ref="A1:O2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="26.08984375" style="2" customWidth="1"/>
+    <col min="2" max="3" width="26.1796875" style="2" customWidth="1"/>
+    <col min="4" max="4" width="17.81640625" style="2" customWidth="1"/>
+    <col min="5" max="5" width="17.453125" style="2" customWidth="1"/>
+    <col min="6" max="6" width="17.90625" style="2" customWidth="1"/>
+    <col min="7" max="7" width="18.36328125" style="2" customWidth="1"/>
+    <col min="8" max="8" width="8.7265625" style="2"/>
+    <col min="9" max="9" width="17.08984375" style="2" customWidth="1"/>
+    <col min="10" max="10" width="14.453125" style="2" customWidth="1"/>
+    <col min="11" max="11" width="19.6328125" style="2" customWidth="1"/>
+    <col min="12" max="12" width="17.81640625" style="2" customWidth="1"/>
+    <col min="13" max="14" width="17.453125" style="2" customWidth="1"/>
+    <col min="15" max="16384" width="8.7265625" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="K1" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="L1" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="M1" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="N1" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="O1" s="5"/>
+    </row>
+    <row r="2" spans="1:15" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="A2" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="H2" s="2">
+        <v>3</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>238</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:O1" xr:uid="{AD994AD9-DD9F-4AD2-9BE6-CF2C5785A85E}"/>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{A2DE0EB7-AD60-4324-8920-12328C3E6B73}"/>
+    <hyperlink ref="C2" r:id="rId2" xr:uid="{09E9CC2E-6823-446F-944E-E57BE9EFB526}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D90093C-235B-4BFA-AC06-070A87C8F0C6}">
   <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -4169,7 +4442,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C97E19B9-CD82-4865-8D9B-AA4D0F508F84}">
   <dimension ref="A1:N5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -4213,7 +4486,7 @@
         <v>140</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="J1" s="5" t="s">
         <v>44</v>
@@ -4233,37 +4506,37 @@
     </row>
     <row r="2" spans="1:14" s="9" customFormat="1" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A2" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="B2" s="7" t="s">
         <v>217</v>
       </c>
-      <c r="B2" s="7" t="s">
-        <v>218</v>
-      </c>
       <c r="C2" s="5" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="E2" s="9" t="s">
         <v>25</v>
       </c>
       <c r="F2" s="5"/>
       <c r="G2" s="5" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="H2" s="9">
         <v>3</v>
       </c>
       <c r="J2" s="9" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="L2" s="9" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.35">
       <c r="E5" s="9" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
   </sheetData>
@@ -4275,7 +4548,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2BBB5AD9-6759-49B8-8C85-DCC62C1F65FC}">
   <dimension ref="A1:N4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -4321,7 +4594,7 @@
         <v>140</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="J1" s="5" t="s">
         <v>44</v>
@@ -4341,16 +4614,16 @@
     </row>
     <row r="2" spans="1:14" ht="333.5" x14ac:dyDescent="0.35">
       <c r="A2" s="5" t="s">
+        <v>205</v>
+      </c>
+      <c r="B2" s="7" t="s">
         <v>206</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="C2" s="5" t="s">
         <v>207</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="D2" s="5" t="s">
         <v>208</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>209</v>
       </c>
       <c r="E2" s="5" t="s">
         <v>25</v>
@@ -4359,33 +4632,33 @@
         <v>43</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="H2" s="5">
         <v>3</v>
       </c>
       <c r="L2" s="5" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.35">
       <c r="B3" s="7"/>
       <c r="L3" s="5" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="4" spans="1:14" s="9" customFormat="1" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="B4" s="7" t="s">
         <v>217</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="C4" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="D4" s="5" t="s">
         <v>219</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>220</v>
       </c>
       <c r="E4" s="9" t="s">
         <v>25</v>
@@ -4394,16 +4667,16 @@
         <v>66</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="H4" s="9">
         <v>3</v>
       </c>
       <c r="J4" s="9" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="L4" s="9" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
sloved bridges in the graph and articulation nodes in the graph
</commit_message>
<xml_diff>
--- a/DSA.xlsx
+++ b/DSA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\2026\learninglog\DSA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CF39B83-41BE-4954-AF76-DB6D15D14AD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BBAD9D4-9CC8-4F2A-A828-ABFD3FF1BD1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,19 +18,20 @@
     <sheet name="Recurrsion" sheetId="3" r:id="rId3"/>
     <sheet name="Tree" sheetId="4" r:id="rId4"/>
     <sheet name="Graph" sheetId="5" r:id="rId5"/>
-    <sheet name="Bitmanupulation" sheetId="9" r:id="rId6"/>
-    <sheet name="LinkedList" sheetId="6" r:id="rId7"/>
-    <sheet name="Subarray" sheetId="8" r:id="rId8"/>
-    <sheet name="Sliding Window" sheetId="7" r:id="rId9"/>
+    <sheet name="DP" sheetId="10" r:id="rId6"/>
+    <sheet name="Bitmanupulation" sheetId="9" r:id="rId7"/>
+    <sheet name="LinkedList" sheetId="6" r:id="rId8"/>
+    <sheet name="Subarray" sheetId="8" r:id="rId9"/>
+    <sheet name="Sliding Window" sheetId="7" r:id="rId10"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Bitmanupulation!$A$1:$O$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">Bitmanupulation!$A$1:$O$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">DP!$A$1:$O$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Graph!$A$1:$N$32</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Sliding Window'!$A$1:$O$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">Subarray!$A$1:$N$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Sliding Window'!$A$1:$O$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">Subarray!$A$1:$N$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="538" uniqueCount="270">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="594" uniqueCount="289">
   <si>
     <t xml:space="preserve">Problem Name </t>
   </si>
@@ -2470,11 +2471,20 @@
     <t>https://leetcode.com/problems/most-stones-removed-with-same-row-or-column</t>
   </si>
   <si>
+    <t>TC - O(N · α(N))</t>
+  </si>
+  <si>
+    <t>Medium-hard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">yes - must visit / striver's video </t>
+  </si>
+  <si>
     <t>Intutions : If we treat each stone’s (row, col) as connected via row or column, stones sharing the same row or column belong to the same component.
 Approch : 
 n^2 - 
 - Treat each coordinate as a vertex.
-- Create edges between vertices having same row or same column.
+- "Create edges" between vertices having same row or same column. (n^2)
 - Process edges using Disjoint Set.
 - Count distinct ultimate parents.
 ans = total_vertices − components.
@@ -2490,13 +2500,146 @@
  - ans = stones − components.</t>
   </si>
   <si>
-    <t>TC - O(N · α(N))</t>
-  </si>
-  <si>
-    <t>Medium-hard</t>
-  </si>
-  <si>
-    <t xml:space="preserve">yes - must visit / striver's video </t>
+    <t>https://leetcode.com/problems/accounts-merge/</t>
+  </si>
+  <si>
+    <t>721. Accounts Merge</t>
+  </si>
+  <si>
+    <t>Intution : If we consider  both person's (indexes) belong to the same component if they have an similar email between them . Then by applying disjoint set we can merge emails easily . 
+Note - Challenge was to find email belongs to which index / collecting indexs based on the email . TC - O(n^2). 
+Approch - 
+- Iterate over all accounts and map each email → index.
+- If an email is already present in the map:
+--Union the current index with the mapped index.
+- After processing all emails, DSU will have formed the components.
+- Create a map: parent → list of emails.
+- For each email:
+-- Find its ultimate parent (account index). (to process all the emails of two different indexes  0 -&gt; j1 , j2 , 1 - j1 , "j5")
+-- Add the email to that parent’s group.
+- Sort emails in each group and return the result.</t>
+  </si>
+  <si>
+    <t>TC -  O(N+E) + O(E*4ɑ) + O(N*(ElogE + E)) where N = no. of indices or nodes and E = no. of emails. The first term is for visiting all the emails. The second term is for merging the accounts. And the third term is for sorting the emails and storing them in the answer array.
+SC - O(N)</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/making-a-large-island/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">827. Making A Large Island - 
+Can convert at most one 0-cell to 1-cell . Return largest island can we create </t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Intution : Treat each cell as a node and form connected components of 1s using DSU.
+If we flip a 0 → 1, it can connect multiple adjacent components, so the new island size becomes the sum of distinct neighboring component sizes + 1.
+How to represent I,J in size , parent = I,J = I*n(lengthofcolumn)+J.
+Approch : 
+- Represent (i, j) as a node: node = i * n + j. 
+- Initialize DSU with n*n nodes.
+- For each cell with value 1: do union with all 4 adjacents and fill parent and size array . 
+- Initialize largestIsland .
+- Try flipping each 0
+- For every cell where grid[i][j] == 0:
+- </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Collect distinct ultimate parents of adjacent 1 cells using a HashSet. 
+Why ? suppose grid as - 
+11
+01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+- Sum their sizes:
+- newSize = 1 + sum(size[parent])
+- compare with largestIsland 
+Update maximum answer.</t>
+    </r>
+  </si>
+  <si>
+    <t>O(n^2 α(N^2))</t>
+  </si>
+  <si>
+    <t>1594. Maximum Non Negative Product in a Matrix</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/maximum-non-negative-product-in-a-matrix</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Intution: When traversing the grid to find the maximum product, we encounter a unique challenge that doesn't exist in "maximum sum" problems: Negative Numbers.
+A positive number multiplied by a large positive number stays large.
+A negative number multiplied by a very small negative number can become a very large positive number.
+Because of this "flip" property, we cannot simply keep track of the maximum product at each cell. We must also track the minimum product (the most negative value), as it has the potential to become the maximum product later if it encounters another negative integer.
+max[i][j] = best possible product from here
+min[i][j] = worst (most negative) product from here
+Approch : 
+- Use 2 dp table min and max .
+- intiliaze them with max and min values . 
+- at each steps - calculate max and min value by comparing with  down and right calls . 
+- return max[0][0] as answer </t>
+  </si>
+  <si>
+    <t xml:space="preserve">DP </t>
+  </si>
+  <si>
+    <t>TC - O(M*N) - expoential (2^m+n) but as we are using memo - (m*n)</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/critical-connections-in-a-network</t>
+  </si>
+  <si>
+    <t>TC - O(V+E)
+SC - O(V)</t>
+  </si>
+  <si>
+    <t>Tarjan's Algorithm</t>
+  </si>
+  <si>
+    <t>1192. Critical Connections in a Network - Tarjan's Algorithm</t>
+  </si>
+  <si>
+    <t>INTUTION : If a child node can't reach any node visited before its parent . (i.e., no back-edge exists),
+then the edge connecting parent → child is a CRITICAL CONNECTION.
+APPROCH : 
+-  Maintain two arrays:
+  insertionTime[n], low[n]  // (minInsertionOfChildsCanReach)
+- Start DFS from any node.
+- Maintain a global timer (initially 1).
+- During DFS for a node:
+- Set:
+insertionTime[node] = low[node] = timer
+do - timer++
+- For each neighbor:
+- if neighbor == parent then continue;
+- If neighbor is not visited:
+-- Call DFS(neighbor, node)
+Update:
+low[node] = min(low[node], low[neighbor])
+- this tells us if we are visiting any previous node which is already visited if its visited will get low[neighbor]&lt;low[node].
+- After visiting a node completly
+- Check for bridge between:
+if (low[neighbor] &gt; insertionTime[node])
+→ edge (node, neighbor) is a bridge .</t>
+  </si>
+  <si>
+    <t>G-56. Articulation Point in Graph</t>
   </si>
 </sst>
 </file>
@@ -2613,9 +2756,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -2629,6 +2769,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2991,6 +3134,147 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2BBB5AD9-6759-49B8-8C85-DCC62C1F65FC}">
+  <dimension ref="A1:N4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="25.6328125" style="5" customWidth="1"/>
+    <col min="2" max="2" width="26.1796875" style="5" customWidth="1"/>
+    <col min="3" max="3" width="25.7265625" style="5" customWidth="1"/>
+    <col min="4" max="4" width="18" style="5" customWidth="1"/>
+    <col min="5" max="5" width="17.7265625" style="5" customWidth="1"/>
+    <col min="6" max="6" width="17.90625" style="5" customWidth="1"/>
+    <col min="7" max="7" width="17.54296875" style="5" customWidth="1"/>
+    <col min="8" max="8" width="19.26953125" style="5" customWidth="1"/>
+    <col min="9" max="9" width="17.81640625" style="2" customWidth="1"/>
+    <col min="10" max="10" width="17.6328125" style="2" customWidth="1"/>
+    <col min="11" max="11" width="17.54296875" style="2" customWidth="1"/>
+    <col min="12" max="12" width="17.1796875" style="5" customWidth="1"/>
+    <col min="13" max="16384" width="8.7265625" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" s="5" customFormat="1" ht="29" x14ac:dyDescent="0.35">
+      <c r="A1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="K1" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="L1" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="M1" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="N1" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" ht="333.5" x14ac:dyDescent="0.35">
+      <c r="A2" s="5" t="s">
+        <v>205</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>206</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="H2" s="5">
+        <v>3</v>
+      </c>
+      <c r="L2" s="5" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="B3" s="6"/>
+      <c r="L3" s="5" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" s="8" customFormat="1" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="A4" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>217</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="H4" s="8">
+        <v>3</v>
+      </c>
+      <c r="J4" s="8" t="s">
+        <v>213</v>
+      </c>
+      <c r="L4" s="8" t="s">
+        <v>221</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:O1" xr:uid="{2BBB5AD9-6759-49B8-8C85-DCC62C1F65FC}"/>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{78E200A1-F1DC-4FA8-ACD2-EB3A411CCC64}"/>
+    <hyperlink ref="B4" r:id="rId2" xr:uid="{A45A0E55-7AB9-485C-AA0D-19E5272C99AD}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE9EF021-EC0E-48FF-9C7E-A5FF2E79A8F1}">
   <dimension ref="A1:L2"/>
@@ -3277,21 +3561,21 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{627F4D11-A7C4-43BB-9B31-F105D2E4CA7B}">
-  <dimension ref="A1:O36"/>
+  <dimension ref="A1:O47"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="25.90625" style="5" customWidth="1"/>
     <col min="2" max="2" width="43.26953125" style="5" customWidth="1"/>
     <col min="3" max="3" width="27.7265625" style="5" customWidth="1"/>
     <col min="4" max="4" width="26.26953125" style="5" customWidth="1"/>
-    <col min="5" max="5" width="17.7265625" style="9" customWidth="1"/>
-    <col min="6" max="6" width="17.6328125" style="9" customWidth="1"/>
+    <col min="5" max="5" width="17.7265625" style="8" customWidth="1"/>
+    <col min="6" max="6" width="17.6328125" style="8" customWidth="1"/>
     <col min="7" max="10" width="17.54296875" style="5" customWidth="1"/>
-    <col min="11" max="11" width="17.453125" style="9" customWidth="1"/>
+    <col min="11" max="11" width="17.453125" style="8" customWidth="1"/>
     <col min="12" max="12" width="17.453125" style="5" customWidth="1"/>
     <col min="13" max="13" width="17.54296875" style="5" customWidth="1"/>
-    <col min="14" max="14" width="17.6328125" style="9" customWidth="1"/>
-    <col min="15" max="15" width="8.7265625" style="9"/>
+    <col min="14" max="14" width="17.6328125" style="8" customWidth="1"/>
+    <col min="15" max="15" width="8.7265625" style="8"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="29" x14ac:dyDescent="0.35">
@@ -3310,7 +3594,7 @@
       <c r="E1" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="F1" s="8" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="5" t="s">
@@ -3342,7 +3626,7 @@
       <c r="A2" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="6" t="s">
         <v>37</v>
       </c>
       <c r="C2" s="5" t="s">
@@ -3351,10 +3635,10 @@
       <c r="D2" s="5" t="s">
         <v>154</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="F2" s="9" t="s">
+      <c r="F2" s="8" t="s">
         <v>39</v>
       </c>
       <c r="G2" s="5" t="s">
@@ -3369,7 +3653,7 @@
       <c r="J2" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="K2" s="9" t="s">
+      <c r="K2" s="8" t="s">
         <v>49</v>
       </c>
       <c r="M2" s="5" t="s">
@@ -3380,7 +3664,7 @@
       <c r="A3" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="6" t="s">
         <v>137</v>
       </c>
       <c r="C3" s="5" t="s">
@@ -3407,7 +3691,7 @@
       <c r="J3" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="K3" s="9" t="s">
+      <c r="K3" s="8" t="s">
         <v>32</v>
       </c>
     </row>
@@ -3415,19 +3699,19 @@
       <c r="A4" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="7" t="s">
         <v>148</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="E4" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="F4" s="9" t="s">
+      <c r="F4" s="8" t="s">
         <v>33</v>
       </c>
       <c r="G4" s="5" t="s">
@@ -3442,7 +3726,7 @@
       <c r="J4" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="K4" s="9" t="s">
+      <c r="K4" s="8" t="s">
         <v>49</v>
       </c>
     </row>
@@ -3450,7 +3734,7 @@
       <c r="A5" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="6" t="s">
         <v>146</v>
       </c>
       <c r="C5" s="5" t="s">
@@ -3459,10 +3743,10 @@
       <c r="D5" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="E5" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="F5" s="9" t="s">
+      <c r="F5" s="8" t="s">
         <v>43</v>
       </c>
       <c r="G5" s="5" t="s">
@@ -3474,7 +3758,7 @@
       <c r="I5" s="5" t="s">
         <v>199</v>
       </c>
-      <c r="K5" s="9" t="s">
+      <c r="K5" s="8" t="s">
         <v>49</v>
       </c>
       <c r="M5" s="5" t="s">
@@ -3485,7 +3769,7 @@
       <c r="A6" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="6" t="s">
         <v>46</v>
       </c>
       <c r="C6" s="5" t="s">
@@ -3494,10 +3778,10 @@
       <c r="D6" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="E6" s="9" t="s">
+      <c r="E6" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="F6" s="9" t="s">
+      <c r="F6" s="8" t="s">
         <v>33</v>
       </c>
       <c r="G6" s="5" t="s">
@@ -3509,7 +3793,7 @@
       <c r="I6" s="5" t="s">
         <v>199</v>
       </c>
-      <c r="K6" s="9" t="s">
+      <c r="K6" s="8" t="s">
         <v>49</v>
       </c>
       <c r="M6" s="5" t="s">
@@ -3520,10 +3804,10 @@
       <c r="A7" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="C7" s="10" t="s">
+      <c r="C7" s="9" t="s">
         <v>195</v>
       </c>
       <c r="D7" s="5" t="s">
@@ -3555,10 +3839,10 @@
       </c>
     </row>
     <row r="8" spans="1:14" ht="232" x14ac:dyDescent="0.35">
-      <c r="A8" s="6" t="s">
+      <c r="A8" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="6" t="s">
         <v>62</v>
       </c>
       <c r="C8" s="5" t="s">
@@ -3567,10 +3851,10 @@
       <c r="D8" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="E8" s="9" t="s">
+      <c r="E8" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="F8" s="9" t="s">
+      <c r="F8" s="8" t="s">
         <v>43</v>
       </c>
       <c r="G8" s="5" t="s">
@@ -3590,7 +3874,7 @@
       <c r="A9" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="6" t="s">
         <v>65</v>
       </c>
       <c r="C9" s="5" t="s">
@@ -3599,10 +3883,10 @@
       <c r="D9" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="E9" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="F9" s="9" t="s">
+      <c r="F9" s="8" t="s">
         <v>66</v>
       </c>
       <c r="G9" s="5" t="s">
@@ -3654,7 +3938,7 @@
       <c r="A11" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="6" t="s">
         <v>76</v>
       </c>
       <c r="C11" s="5" t="s">
@@ -3663,10 +3947,10 @@
       <c r="D11" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="E11" s="9" t="s">
+      <c r="E11" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="F11" s="9" t="s">
+      <c r="F11" s="8" t="s">
         <v>60</v>
       </c>
       <c r="G11" s="5" t="s">
@@ -3695,10 +3979,10 @@
       <c r="D12" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="E12" s="9" t="s">
+      <c r="E12" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="F12" s="9" t="s">
+      <c r="F12" s="8" t="s">
         <v>43</v>
       </c>
       <c r="G12" s="5" t="s">
@@ -3753,7 +4037,7 @@
       <c r="A14" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="6" t="s">
         <v>98</v>
       </c>
       <c r="C14" s="5" t="s">
@@ -3785,7 +4069,7 @@
       <c r="A15" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="B15" s="6" t="s">
         <v>102</v>
       </c>
       <c r="C15" s="5" t="s">
@@ -3849,7 +4133,7 @@
       <c r="A17" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="B17" s="7" t="s">
+      <c r="B17" s="6" t="s">
         <v>120</v>
       </c>
       <c r="C17" s="5" t="s">
@@ -3951,19 +4235,19 @@
       <c r="A20" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="B20" s="7" t="s">
+      <c r="B20" s="6" t="s">
         <v>157</v>
       </c>
-      <c r="C20" s="10" t="s">
+      <c r="C20" s="9" t="s">
         <v>152</v>
       </c>
       <c r="D20" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="E20" s="9" t="s">
+      <c r="E20" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="F20" s="9" t="s">
+      <c r="F20" s="8" t="s">
         <v>43</v>
       </c>
       <c r="G20" s="5" t="s">
@@ -3975,7 +4259,7 @@
       <c r="I20" s="5" t="s">
         <v>197</v>
       </c>
-      <c r="K20" s="9" t="s">
+      <c r="K20" s="8" t="s">
         <v>32</v>
       </c>
       <c r="L20" s="5" t="s">
@@ -3989,7 +4273,7 @@
       <c r="A21" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="B21" s="7" t="s">
+      <c r="B21" s="6" t="s">
         <v>157</v>
       </c>
       <c r="C21" s="5" t="s">
@@ -3998,10 +4282,10 @@
       <c r="D21" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="E21" s="9" t="s">
+      <c r="E21" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="F21" s="9" t="s">
+      <c r="F21" s="8" t="s">
         <v>138</v>
       </c>
       <c r="G21" s="5" t="s">
@@ -4010,7 +4294,7 @@
       <c r="H21" s="5">
         <v>4</v>
       </c>
-      <c r="K21" s="9" t="s">
+      <c r="K21" s="8" t="s">
         <v>32</v>
       </c>
       <c r="L21" s="5" t="s">
@@ -4030,10 +4314,10 @@
       <c r="D22" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="E22" s="9" t="s">
+      <c r="E22" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="F22" s="9" t="s">
+      <c r="F22" s="8" t="s">
         <v>43</v>
       </c>
       <c r="G22" s="5" t="s">
@@ -4042,7 +4326,7 @@
       <c r="H22" s="5">
         <v>4</v>
       </c>
-      <c r="K22" s="9" t="s">
+      <c r="K22" s="8" t="s">
         <v>32</v>
       </c>
       <c r="L22" s="5" t="s">
@@ -4056,19 +4340,19 @@
       <c r="A23" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="B23" s="7" t="s">
+      <c r="B23" s="6" t="s">
         <v>172</v>
       </c>
-      <c r="C23" s="10" t="s">
+      <c r="C23" s="9" t="s">
         <v>179</v>
       </c>
       <c r="D23" s="5" t="s">
         <v>214</v>
       </c>
-      <c r="E23" s="9" t="s">
+      <c r="E23" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="F23" s="9" t="s">
+      <c r="F23" s="8" t="s">
         <v>43</v>
       </c>
       <c r="G23" s="5" t="s">
@@ -4077,7 +4361,7 @@
       <c r="H23" s="5">
         <v>3</v>
       </c>
-      <c r="K23" s="9" t="s">
+      <c r="K23" s="8" t="s">
         <v>32</v>
       </c>
       <c r="L23" s="5" t="s">
@@ -4088,7 +4372,7 @@
       <c r="A24" s="5" t="s">
         <v>176</v>
       </c>
-      <c r="B24" s="7" t="s">
+      <c r="B24" s="6" t="s">
         <v>177</v>
       </c>
       <c r="C24" s="5" t="s">
@@ -4097,10 +4381,10 @@
       <c r="D24" s="5" t="s">
         <v>173</v>
       </c>
-      <c r="E24" s="9" t="s">
+      <c r="E24" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="F24" s="9" t="s">
+      <c r="F24" s="8" t="s">
         <v>43</v>
       </c>
       <c r="G24" s="5" t="s">
@@ -4109,7 +4393,7 @@
       <c r="H24" s="5">
         <v>3</v>
       </c>
-      <c r="K24" s="9" t="s">
+      <c r="K24" s="8" t="s">
         <v>32</v>
       </c>
       <c r="L24" s="5" t="s">
@@ -4120,7 +4404,7 @@
       <c r="A25" s="5" t="s">
         <v>180</v>
       </c>
-      <c r="B25" s="7" t="s">
+      <c r="B25" s="6" t="s">
         <v>181</v>
       </c>
       <c r="C25" s="5" t="s">
@@ -4129,10 +4413,10 @@
       <c r="D25" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="E25" s="9" t="s">
+      <c r="E25" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="F25" s="9" t="s">
+      <c r="F25" s="8" t="s">
         <v>43</v>
       </c>
       <c r="G25" s="5" t="s">
@@ -4141,7 +4425,7 @@
       <c r="H25" s="5">
         <v>3</v>
       </c>
-      <c r="K25" s="9" t="s">
+      <c r="K25" s="8" t="s">
         <v>32</v>
       </c>
     </row>
@@ -4149,7 +4433,7 @@
       <c r="A26" s="5" t="s">
         <v>185</v>
       </c>
-      <c r="B26" s="7" t="s">
+      <c r="B26" s="6" t="s">
         <v>186</v>
       </c>
       <c r="C26" s="5" t="s">
@@ -4158,10 +4442,10 @@
       <c r="D26" s="5" t="s">
         <v>188</v>
       </c>
-      <c r="E26" s="9" t="s">
+      <c r="E26" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="F26" s="9" t="s">
+      <c r="F26" s="8" t="s">
         <v>43</v>
       </c>
       <c r="G26" s="5" t="s">
@@ -4170,7 +4454,7 @@
       <c r="H26" s="5">
         <v>3</v>
       </c>
-      <c r="K26" s="9" t="s">
+      <c r="K26" s="8" t="s">
         <v>32</v>
       </c>
       <c r="L26" s="5" t="s">
@@ -4181,7 +4465,7 @@
       <c r="A27" s="5" t="s">
         <v>190</v>
       </c>
-      <c r="B27" s="7" t="s">
+      <c r="B27" s="6" t="s">
         <v>191</v>
       </c>
       <c r="C27" s="5" t="s">
@@ -4190,10 +4474,10 @@
       <c r="D27" s="5" t="s">
         <v>193</v>
       </c>
-      <c r="E27" s="9" t="s">
+      <c r="E27" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="F27" s="9" t="s">
+      <c r="F27" s="8" t="s">
         <v>43</v>
       </c>
       <c r="G27" s="5" t="s">
@@ -4205,7 +4489,7 @@
       <c r="I27" s="5" t="s">
         <v>242</v>
       </c>
-      <c r="K27" s="9" t="s">
+      <c r="K27" s="8" t="s">
         <v>32</v>
       </c>
       <c r="L27" s="5" t="s">
@@ -4219,7 +4503,7 @@
       <c r="A28" s="5" t="s">
         <v>200</v>
       </c>
-      <c r="B28" s="7" t="s">
+      <c r="B28" s="6" t="s">
         <v>201</v>
       </c>
       <c r="C28" s="5" t="s">
@@ -4228,10 +4512,10 @@
       <c r="D28" s="5" t="s">
         <v>202</v>
       </c>
-      <c r="E28" s="9" t="s">
+      <c r="E28" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="F28" s="9" t="s">
+      <c r="F28" s="8" t="s">
         <v>203</v>
       </c>
       <c r="G28" s="5" t="s">
@@ -4243,7 +4527,7 @@
       <c r="I28" s="5" t="s">
         <v>240</v>
       </c>
-      <c r="K28" s="9" t="s">
+      <c r="K28" s="8" t="s">
         <v>32</v>
       </c>
       <c r="L28" s="5" t="s">
@@ -4257,7 +4541,7 @@
       <c r="A29" s="5" t="s">
         <v>210</v>
       </c>
-      <c r="B29" s="7" t="s">
+      <c r="B29" s="6" t="s">
         <v>211</v>
       </c>
       <c r="C29" s="5" t="s">
@@ -4266,10 +4550,10 @@
       <c r="D29" s="5" t="s">
         <v>212</v>
       </c>
-      <c r="E29" s="9" t="s">
+      <c r="E29" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="F29" s="9" t="s">
+      <c r="F29" s="8" t="s">
         <v>66</v>
       </c>
       <c r="G29" s="5" t="s">
@@ -4289,19 +4573,19 @@
       <c r="A30" s="5" t="s">
         <v>226</v>
       </c>
-      <c r="B30" s="7" t="s">
+      <c r="B30" s="6" t="s">
         <v>225</v>
       </c>
-      <c r="C30" s="11" t="s">
+      <c r="C30" s="10" t="s">
         <v>227</v>
       </c>
       <c r="D30" s="5" t="s">
         <v>228</v>
       </c>
-      <c r="E30" s="9" t="s">
+      <c r="E30" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="F30" s="9" t="s">
+      <c r="F30" s="8" t="s">
         <v>43</v>
       </c>
       <c r="H30" s="5">
@@ -4315,7 +4599,7 @@
       <c r="A31" s="5" t="s">
         <v>229</v>
       </c>
-      <c r="B31" s="7" t="s">
+      <c r="B31" s="6" t="s">
         <v>230</v>
       </c>
       <c r="C31" s="5" t="s">
@@ -4324,10 +4608,10 @@
       <c r="D31" s="5" t="s">
         <v>232</v>
       </c>
-      <c r="E31" s="9" t="s">
+      <c r="E31" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="F31" s="9" t="s">
+      <c r="F31" s="8" t="s">
         <v>43</v>
       </c>
       <c r="G31" s="5" t="s">
@@ -4353,7 +4637,7 @@
       <c r="D32" s="5" t="s">
         <v>246</v>
       </c>
-      <c r="F32" s="9" t="s">
+      <c r="F32" s="8" t="s">
         <v>244</v>
       </c>
       <c r="H32" s="5">
@@ -4376,10 +4660,10 @@
       <c r="D33" s="5" t="s">
         <v>251</v>
       </c>
-      <c r="E33" s="9" t="s">
+      <c r="E33" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="F33" s="9" t="s">
+      <c r="F33" s="8" t="s">
         <v>43</v>
       </c>
       <c r="G33" s="5" t="s">
@@ -4388,7 +4672,7 @@
       <c r="H33" s="5">
         <v>3</v>
       </c>
-      <c r="K33" s="9" t="s">
+      <c r="K33" s="8" t="s">
         <v>32</v>
       </c>
       <c r="L33" s="5" t="s">
@@ -4402,7 +4686,7 @@
       <c r="A34" s="5" t="s">
         <v>254</v>
       </c>
-      <c r="B34" s="7" t="s">
+      <c r="B34" s="6" t="s">
         <v>253</v>
       </c>
       <c r="C34" s="5" t="s">
@@ -4411,10 +4695,10 @@
       <c r="D34" s="5" t="s">
         <v>255</v>
       </c>
-      <c r="E34" s="9" t="s">
+      <c r="E34" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="F34" s="9" t="s">
+      <c r="F34" s="8" t="s">
         <v>43</v>
       </c>
       <c r="G34" s="5" t="s">
@@ -4426,7 +4710,7 @@
       <c r="J34" s="5" t="s">
         <v>257</v>
       </c>
-      <c r="K34" s="9" t="s">
+      <c r="K34" s="8" t="s">
         <v>32</v>
       </c>
     </row>
@@ -4443,10 +4727,10 @@
       <c r="D35" s="5" t="s">
         <v>262</v>
       </c>
-      <c r="E35" s="9" t="s">
+      <c r="E35" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="F35" s="9" t="s">
+      <c r="F35" s="8" t="s">
         <v>43</v>
       </c>
       <c r="G35" s="5" t="s">
@@ -4458,7 +4742,7 @@
       <c r="J35" s="5" t="s">
         <v>263</v>
       </c>
-      <c r="K35" s="9" t="s">
+      <c r="K35" s="8" t="s">
         <v>32</v>
       </c>
       <c r="L35" s="5" t="s">
@@ -4476,16 +4760,16 @@
         <v>265</v>
       </c>
       <c r="C36" s="5" t="s">
+        <v>269</v>
+      </c>
+      <c r="D36" s="5" t="s">
         <v>266</v>
       </c>
-      <c r="D36" s="5" t="s">
+      <c r="E36" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="F36" s="8" t="s">
         <v>267</v>
-      </c>
-      <c r="E36" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="F36" s="9" t="s">
-        <v>268</v>
       </c>
       <c r="G36" s="5" t="s">
         <v>256</v>
@@ -4494,9 +4778,9 @@
         <v>3</v>
       </c>
       <c r="J36" s="5" t="s">
-        <v>269</v>
-      </c>
-      <c r="K36" s="9" t="s">
+        <v>268</v>
+      </c>
+      <c r="K36" s="8" t="s">
         <v>32</v>
       </c>
       <c r="L36" s="5" t="s">
@@ -4504,6 +4788,130 @@
       </c>
       <c r="M36" s="5" t="s">
         <v>254</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="A37" s="5" t="s">
+        <v>271</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>270</v>
+      </c>
+      <c r="C37" s="5" t="s">
+        <v>272</v>
+      </c>
+      <c r="D37" s="5" t="s">
+        <v>273</v>
+      </c>
+      <c r="E37" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="F37" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="G37" s="5" t="s">
+        <v>256</v>
+      </c>
+      <c r="H37" s="5">
+        <v>3</v>
+      </c>
+      <c r="J37" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="K37" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="L37" s="5" t="s">
+        <v>254</v>
+      </c>
+      <c r="M37" s="5" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="A38" s="5" t="s">
+        <v>275</v>
+      </c>
+      <c r="B38" s="5" t="s">
+        <v>274</v>
+      </c>
+      <c r="C38" s="5" t="s">
+        <v>276</v>
+      </c>
+      <c r="D38" s="5" t="s">
+        <v>277</v>
+      </c>
+      <c r="E38" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="F38" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="G38" s="5" t="s">
+        <v>256</v>
+      </c>
+      <c r="H38" s="5">
+        <v>3</v>
+      </c>
+      <c r="J38" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="K38" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="L38" s="5" t="s">
+        <v>254</v>
+      </c>
+      <c r="M38" s="5" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="39" spans="1:13" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="A39" s="5" t="s">
+        <v>286</v>
+      </c>
+      <c r="B39" s="5" t="s">
+        <v>283</v>
+      </c>
+      <c r="C39" s="5" t="s">
+        <v>287</v>
+      </c>
+      <c r="D39" s="5" t="s">
+        <v>284</v>
+      </c>
+      <c r="E39" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="F39" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="G39" s="5" t="s">
+        <v>285</v>
+      </c>
+      <c r="H39" s="5">
+        <v>3</v>
+      </c>
+      <c r="J39" s="5" t="s">
+        <v>213</v>
+      </c>
+      <c r="K39" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="L39" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="M39" s="5" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="40" spans="1:13" ht="29" x14ac:dyDescent="0.35">
+      <c r="A40" s="5" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="47" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="C47" s="5" t="s">
+        <v>214</v>
       </c>
     </row>
   </sheetData>
@@ -4533,13 +4941,110 @@
     <hyperlink ref="B31" r:id="rId22" xr:uid="{3472C449-0813-4249-A912-7371C1132D75}"/>
     <hyperlink ref="B27" r:id="rId23" xr:uid="{E7B363CE-2ADD-4EB8-BDCC-4504C7B2FC63}"/>
     <hyperlink ref="B34" r:id="rId24" xr:uid="{878B70B8-85D8-488D-988D-D9EA1E0D237C}"/>
+    <hyperlink ref="B37" r:id="rId25" xr:uid="{B22C8E31-8548-4614-AF2C-D50B2AEDD07A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId25"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId26"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{520716B6-7F22-460B-B807-1EABD72CDD3C}">
+  <dimension ref="A1:N2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="26.54296875" style="5" customWidth="1"/>
+    <col min="2" max="2" width="26.26953125" style="5" customWidth="1"/>
+    <col min="3" max="3" width="26.08984375" style="5" customWidth="1"/>
+    <col min="4" max="4" width="17.36328125" style="5" customWidth="1"/>
+    <col min="5" max="5" width="17.54296875" style="5" customWidth="1"/>
+    <col min="6" max="6" width="17.90625" style="5" customWidth="1"/>
+    <col min="7" max="7" width="17.6328125" style="5" customWidth="1"/>
+    <col min="8" max="8" width="8.7265625" style="5"/>
+    <col min="9" max="9" width="17.6328125" style="5" customWidth="1"/>
+    <col min="10" max="16384" width="8.7265625" style="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="K1" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="L1" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="M1" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="N1" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="A2" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>279</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>280</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>282</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>281</v>
+      </c>
+      <c r="H2" s="5">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:O1" xr:uid="{520716B6-7F22-460B-B807-1EABD72CDD3C}"/>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{919D73E7-9EA6-43E1-B38C-FE27D065BFAD}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD994AD9-DD9F-4AD2-9BE6-CF2C5785A85E}">
   <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -4643,25 +5148,25 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D90093C-235B-4BFA-AC06-070A87C8F0C6}">
   <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="40.36328125" style="9" customWidth="1"/>
+    <col min="1" max="1" width="40.36328125" style="8" customWidth="1"/>
     <col min="2" max="2" width="31" style="5" customWidth="1"/>
     <col min="3" max="3" width="28.36328125" style="5" customWidth="1"/>
-    <col min="4" max="4" width="16.36328125" style="9" customWidth="1"/>
-    <col min="5" max="5" width="18.26953125" style="9" customWidth="1"/>
-    <col min="6" max="6" width="17.54296875" style="9" customWidth="1"/>
-    <col min="7" max="7" width="19.26953125" style="9" customWidth="1"/>
-    <col min="8" max="8" width="21.90625" style="9" customWidth="1"/>
-    <col min="9" max="9" width="18.453125" style="9" customWidth="1"/>
-    <col min="10" max="10" width="21.7265625" style="9" customWidth="1"/>
+    <col min="4" max="4" width="16.36328125" style="8" customWidth="1"/>
+    <col min="5" max="5" width="18.26953125" style="8" customWidth="1"/>
+    <col min="6" max="6" width="17.54296875" style="8" customWidth="1"/>
+    <col min="7" max="7" width="19.26953125" style="8" customWidth="1"/>
+    <col min="8" max="8" width="21.90625" style="8" customWidth="1"/>
+    <col min="9" max="9" width="18.453125" style="8" customWidth="1"/>
+    <col min="10" max="10" width="21.7265625" style="8" customWidth="1"/>
     <col min="11" max="11" width="17" customWidth="1"/>
     <col min="12" max="12" width="17.453125" style="5" customWidth="1"/>
     <col min="13" max="13" width="17.26953125" style="5" customWidth="1"/>
-    <col min="14" max="14" width="17.36328125" style="9" customWidth="1"/>
+    <col min="14" max="14" width="17.36328125" style="8" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="29" x14ac:dyDescent="0.35">
@@ -4680,7 +5185,7 @@
       <c r="E1" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="F1" s="8" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="5" t="s">
@@ -4707,40 +5212,40 @@
       <c r="N1" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="O1" s="9"/>
+      <c r="O1" s="8"/>
     </row>
     <row r="2" spans="1:15" ht="409.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="8" t="s">
         <v>160</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="6" t="s">
         <v>161</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>166</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="D2" s="8" t="s">
         <v>162</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="F2" s="9" t="s">
+      <c r="F2" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="G2" s="9" t="s">
+      <c r="G2" s="8" t="s">
         <v>163</v>
       </c>
-      <c r="H2" s="9">
+      <c r="H2" s="8">
         <v>3</v>
       </c>
-      <c r="J2" s="9" t="s">
+      <c r="J2" s="8" t="s">
         <v>165</v>
       </c>
-      <c r="L2" s="7" t="s">
+      <c r="L2" s="6" t="s">
         <v>164</v>
       </c>
-      <c r="M2" s="7" t="s">
+      <c r="M2" s="6" t="s">
         <v>164</v>
       </c>
     </row>
@@ -4754,7 +5259,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C97E19B9-CD82-4865-8D9B-AA4D0F508F84}">
   <dimension ref="A1:N5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -4763,11 +5268,11 @@
     <col min="2" max="2" width="17.90625" style="2" customWidth="1"/>
     <col min="3" max="3" width="26" style="5" customWidth="1"/>
     <col min="4" max="4" width="16.81640625" style="5" customWidth="1"/>
-    <col min="5" max="5" width="17.08984375" style="9" customWidth="1"/>
+    <col min="5" max="5" width="17.08984375" style="8" customWidth="1"/>
     <col min="6" max="6" width="17.26953125" style="5" customWidth="1"/>
     <col min="7" max="7" width="16.36328125" customWidth="1"/>
-    <col min="8" max="8" width="21.26953125" style="9" customWidth="1"/>
-    <col min="10" max="10" width="8.7265625" style="9"/>
+    <col min="8" max="8" width="21.26953125" style="8" customWidth="1"/>
+    <col min="10" max="10" width="8.7265625" style="8"/>
     <col min="11" max="11" width="18.26953125" customWidth="1"/>
     <col min="12" max="12" width="17.26953125" customWidth="1"/>
   </cols>
@@ -4816,11 +5321,11 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:14" s="9" customFormat="1" ht="409.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:14" s="8" customFormat="1" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A2" s="5" t="s">
         <v>216</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="6" t="s">
         <v>217</v>
       </c>
       <c r="C2" s="5" t="s">
@@ -4829,25 +5334,25 @@
       <c r="D2" s="5" t="s">
         <v>219</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" s="8" t="s">
         <v>25</v>
       </c>
       <c r="F2" s="5"/>
       <c r="G2" s="5" t="s">
         <v>220</v>
       </c>
-      <c r="H2" s="9">
+      <c r="H2" s="8">
         <v>3</v>
       </c>
-      <c r="J2" s="9" t="s">
+      <c r="J2" s="8" t="s">
         <v>213</v>
       </c>
-      <c r="L2" s="9" t="s">
+      <c r="L2" s="8" t="s">
         <v>222</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="E5" s="9" t="s">
+      <c r="E5" s="8" t="s">
         <v>214</v>
       </c>
     </row>
@@ -4858,145 +5363,4 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2BBB5AD9-6759-49B8-8C85-DCC62C1F65FC}">
-  <dimension ref="A1:N4"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="25.6328125" style="5" customWidth="1"/>
-    <col min="2" max="2" width="26.1796875" style="5" customWidth="1"/>
-    <col min="3" max="3" width="25.7265625" style="5" customWidth="1"/>
-    <col min="4" max="4" width="18" style="5" customWidth="1"/>
-    <col min="5" max="5" width="17.7265625" style="5" customWidth="1"/>
-    <col min="6" max="6" width="17.90625" style="5" customWidth="1"/>
-    <col min="7" max="7" width="17.54296875" style="5" customWidth="1"/>
-    <col min="8" max="8" width="19.26953125" style="5" customWidth="1"/>
-    <col min="9" max="9" width="17.81640625" style="2" customWidth="1"/>
-    <col min="10" max="10" width="17.6328125" style="2" customWidth="1"/>
-    <col min="11" max="11" width="17.54296875" style="2" customWidth="1"/>
-    <col min="12" max="12" width="17.1796875" style="5" customWidth="1"/>
-    <col min="13" max="16384" width="8.7265625" style="2"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:14" s="5" customFormat="1" ht="29" x14ac:dyDescent="0.35">
-      <c r="A1" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="I1" s="5" t="s">
-        <v>196</v>
-      </c>
-      <c r="J1" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="K1" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="L1" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="M1" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="N1" s="5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" ht="333.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="5" t="s">
-        <v>205</v>
-      </c>
-      <c r="B2" s="7" t="s">
-        <v>206</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>207</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>208</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>209</v>
-      </c>
-      <c r="H2" s="5">
-        <v>3</v>
-      </c>
-      <c r="L2" s="5" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="B3" s="7"/>
-      <c r="L3" s="5" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" s="9" customFormat="1" ht="409.5" x14ac:dyDescent="0.35">
-      <c r="A4" s="5" t="s">
-        <v>216</v>
-      </c>
-      <c r="B4" s="7" t="s">
-        <v>217</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>218</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>219</v>
-      </c>
-      <c r="E4" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>220</v>
-      </c>
-      <c r="H4" s="9">
-        <v>3</v>
-      </c>
-      <c r="J4" s="9" t="s">
-        <v>213</v>
-      </c>
-      <c r="L4" s="9" t="s">
-        <v>221</v>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:O1" xr:uid="{2BBB5AD9-6759-49B8-8C85-DCC62C1F65FC}"/>
-  <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1" xr:uid="{78E200A1-F1DC-4FA8-ACD2-EB3A411CCC64}"/>
-    <hyperlink ref="B4" r:id="rId2" xr:uid="{A45A0E55-7AB9-485C-AA0D-19E5272C99AD}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>